<commit_message>
fix(backend): resolve socket test issue
</commit_message>
<xml_diff>
--- a/apps/backend/excel-data/issuereturn_library_migration.xlsx
+++ b/apps/backend/excel-data/issuereturn_library_migration.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4282" uniqueCount="1435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5008" uniqueCount="1678">
   <si>
     <t>legacy_id</t>
   </si>
@@ -4316,6 +4316,736 @@
   </si>
   <si>
     <t>2026-05-11T06:24:39.339Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:28.072Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:32.826Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:35.519Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:41.618Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:44.115Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:46.128Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:47.559Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:49.591Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:51.084Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:52.279Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:54.008Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:55.301Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:56.657Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:57.865Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:46:59.029Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:00.215Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:01.475Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:02.839Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:04.215Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:05.485Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:06.763Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:08.193Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:09.597Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:11.311Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:13.157Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:14.601Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:15.984Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:17.247Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:18.590Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:20.647Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:22.096Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:25.193Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:26.734Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:28.342Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:29.899Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:31.400Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:33.412Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:34.832Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:36.484Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:38.650Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:40.863Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:42.603Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:44.652Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:49.234Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:50.469Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:51.745Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:53.272Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:55.530Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:57.208Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:58.618Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:47:59.783Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:00.982Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:02.472Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:03.568Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:05.141Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:06.247Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:07.570Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:08.910Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:11.288Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:13.002Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:14.347Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:15.785Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:17.799Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:19.152Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:20.257Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:21.896Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:24.757Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:26.260Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:27.960Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:29.705Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:30.863Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:31.934Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:33.052Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:34.390Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:35.529Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:37.153Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:39.774Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:41.928Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:43.785Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:45.566Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:47.081Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:48.680Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:53.264Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:57.074Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:48:59.497Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:02.716Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:08.084Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:14.071Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:16.326Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:17.963Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:19.319Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:20.856Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:22.131Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:23.536Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:24.906Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:26.211Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:27.536Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:28.900Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:30.259Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:31.645Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:33.171Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:34.421Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:35.636Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:37.161Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:38.632Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:41.790Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:44.477Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:48.888Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:53.082Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:56.206Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:49:59.855Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:03.482Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:06.372Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:08.684Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:11.333Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:14.589Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:17.200Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:19.855Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:22.043Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:23.748Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:25.796Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:28.304Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:31.142Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:34.311Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:36.135Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:37.565Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:40.173Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:42.557Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:44.926Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:48.013Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:49.826Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:51.508Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:54.531Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:50:57.981Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:00.213Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:02.387Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:04.062Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:05.611Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:07.079Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:08.756Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:10.791Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:12.934Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:15.550Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:18.511Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:21.022Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:22.862Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:24.502Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:26.087Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:27.379Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:29.008Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:30.353Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:31.822Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:33.473Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:34.820Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:36.569Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:38.318Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:40.566Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:42.524Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:44.871Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:46.317Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:47.845Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:49.187Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:51.495Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:52.858Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:54.383Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:55.642Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:57.054Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:51:58.666Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:00.115Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:01.578Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:03.029Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:04.424Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:06.789Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:10.465Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:12.659Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:14.863Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:17.509Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:19.484Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:22.614Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:24.694Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:27.383Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:29.840Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:31.264Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:32.936Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:34.821Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:36.148Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:37.594Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:38.924Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:40.244Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:41.641Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:52:55.126Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:53:14.385Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:53:27.675Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:53:29.051Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:53:46.449Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:53:59.826Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:54:10.784Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:54:17.076Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:54:25.905Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Failed query: insert into "copy_details" ("id", "legacy_copy_details_id", "book_id_fk", "published_year", "access_number", "old_access_number", "type", "issue_type", "status_id_fk", "entry_mode_id_fk", "rack_id_fk", "shelf_id_fk", "voucher_number", "enclosure_id_fk", "number_of_enclosures", "number_of_pages", "price_in_inr", "price_foreign_currency", "purchase_price", "set_price", "binding_type_id_fk", "isbn", "book_volume", "book_part", "book_part_info", "volume_info", "remarks", "legacy_vendor_id", "donor_person_id_fk", "prefix", "suffix", "pdf_path", "book_size", "bill_date", "discount", "shipping_charges", "created_by_user_id_fk", "created_at", "updated_by_user_id_fk", "updated_at") values (default, $1, $2, $3, $4, $5, $6, $7, $8, $9, $10, $11, $12, default, $13, $14, $15, $16, $17, $18, $19, $20, $21, $22, $23, $24, $25, $26, default, $27, $28, $29, $30, $31, $32, $33, default, $34, default, default) returning "id", "legacy_copy_details_id", "book_id_fk", "published_year", "access_number", "old_access_number", "type", "issue_type", "status_id_fk", "entry_mode_id_fk", "rack_id_fk", "shelf_id_fk", "voucher_number", "enclosure_id_fk", "number_of_enclosures", "number_of_pages", "price_in_inr", "price_foreign_currency", "purchase_price", "set_price", "binding_type_id_fk", "isbn", "book_volume", "book_part", "book_part_info", "volume_info", "remarks", "legacy_vendor_id", "donor_person_id_fk", "prefix", "suffix", "pdf_path", "book_size", "bill_date", "discount", "shipping_charges", "created_by_user_id_fk", "created_at", "updated_by_user_id_fk", "updated_at"
+params: 20473,487,,19793,19793,Text Book,Issue Relevant,1,1,1,26,8932,0,9780571180172,450,0,0,null,1,,,,,,,5,0,0,,,2015-08-13T18:30:00.000Z,0,,2015-08-17T18:30:00.000Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:54:32.364Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:54:38.371Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:54:48.798Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:54:58.053Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:55:05.414Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:55:10.279Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:55:16.131Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:55:17.154Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:55:18.121Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:55:31.345Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:55:38.977Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:55:46.108Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:55:59.740Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:56:07.053Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:56:17.046Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:56:25.094Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:56:26.847Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:56:28.503Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:56:31.068Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:56:33.127Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:56:34.611Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:56:43.827Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:56:53.270Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:57:00.139Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:57:11.343Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:57:22.928Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:57:31.806Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:57:34.041Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:57:47.908Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:57:55.965Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:58:05.272Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:58:16.594Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:58:25.059Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:58:33.515Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:58:45.026Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:58:52.038Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:58:58.459Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:59:06.095Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:59:19.022Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:59:28.759Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:59:41.329Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T07:59:55.051Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:00:15.126Z</t>
   </si>
 </sst>
 </file>
@@ -4696,7 +5426,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1427"/>
+  <dimension ref="A1:D1669"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -24677,6 +25407,3394 @@
         <v>1434</v>
       </c>
     </row>
+    <row r="1428" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1428">
+        <v>36130</v>
+      </c>
+      <c r="B1428" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1428" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1428" t="s">
+        <v>1435</v>
+      </c>
+    </row>
+    <row r="1429" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1429">
+        <v>36982</v>
+      </c>
+      <c r="B1429" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1429" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1429" t="s">
+        <v>1436</v>
+      </c>
+    </row>
+    <row r="1430" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1430">
+        <v>37243</v>
+      </c>
+      <c r="B1430" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1430" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1430" t="s">
+        <v>1437</v>
+      </c>
+    </row>
+    <row r="1431" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1431">
+        <v>38017</v>
+      </c>
+      <c r="B1431" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1431" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1431" t="s">
+        <v>1438</v>
+      </c>
+    </row>
+    <row r="1432" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1432">
+        <v>38021</v>
+      </c>
+      <c r="B1432" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1432" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1432" t="s">
+        <v>1439</v>
+      </c>
+    </row>
+    <row r="1433" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1433">
+        <v>39441</v>
+      </c>
+      <c r="B1433" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1433" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1433" t="s">
+        <v>1440</v>
+      </c>
+    </row>
+    <row r="1434" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1434">
+        <v>39804</v>
+      </c>
+      <c r="B1434" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1434" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1434" t="s">
+        <v>1441</v>
+      </c>
+    </row>
+    <row r="1435" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1435">
+        <v>40721</v>
+      </c>
+      <c r="B1435" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1435" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1435" t="s">
+        <v>1442</v>
+      </c>
+    </row>
+    <row r="1436" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1436">
+        <v>40723</v>
+      </c>
+      <c r="B1436" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1436" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1436" t="s">
+        <v>1443</v>
+      </c>
+    </row>
+    <row r="1437" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1437">
+        <v>40996</v>
+      </c>
+      <c r="B1437" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1437" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1437" t="s">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="1438" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1438">
+        <v>41181</v>
+      </c>
+      <c r="B1438" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1438" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1438" t="s">
+        <v>1445</v>
+      </c>
+    </row>
+    <row r="1439" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1439">
+        <v>41182</v>
+      </c>
+      <c r="B1439" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1439" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1439" t="s">
+        <v>1446</v>
+      </c>
+    </row>
+    <row r="1440" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1440">
+        <v>41696</v>
+      </c>
+      <c r="B1440" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1440" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1440" t="s">
+        <v>1447</v>
+      </c>
+    </row>
+    <row r="1441" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1441">
+        <v>41952</v>
+      </c>
+      <c r="B1441" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1441" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1441" t="s">
+        <v>1448</v>
+      </c>
+    </row>
+    <row r="1442" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1442">
+        <v>41953</v>
+      </c>
+      <c r="B1442" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1442" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1442" t="s">
+        <v>1449</v>
+      </c>
+    </row>
+    <row r="1443" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1443">
+        <v>42439</v>
+      </c>
+      <c r="B1443" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1443" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1443" t="s">
+        <v>1450</v>
+      </c>
+    </row>
+    <row r="1444" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1444">
+        <v>42669</v>
+      </c>
+      <c r="B1444" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1444" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1444" t="s">
+        <v>1451</v>
+      </c>
+    </row>
+    <row r="1445" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1445">
+        <v>42802</v>
+      </c>
+      <c r="B1445" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1445" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1445" t="s">
+        <v>1452</v>
+      </c>
+    </row>
+    <row r="1446" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1446">
+        <v>42854</v>
+      </c>
+      <c r="B1446" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1446" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1446" t="s">
+        <v>1453</v>
+      </c>
+    </row>
+    <row r="1447" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1447">
+        <v>42855</v>
+      </c>
+      <c r="B1447" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1447" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1447" t="s">
+        <v>1454</v>
+      </c>
+    </row>
+    <row r="1448" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1448">
+        <v>43251</v>
+      </c>
+      <c r="B1448" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1448" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1448" t="s">
+        <v>1455</v>
+      </c>
+    </row>
+    <row r="1449" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1449">
+        <v>43620</v>
+      </c>
+      <c r="B1449" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1449" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1449" t="s">
+        <v>1456</v>
+      </c>
+    </row>
+    <row r="1450" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1450">
+        <v>43622</v>
+      </c>
+      <c r="B1450" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1450" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1450" t="s">
+        <v>1457</v>
+      </c>
+    </row>
+    <row r="1451" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1451">
+        <v>44376</v>
+      </c>
+      <c r="B1451" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1451" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1451" t="s">
+        <v>1458</v>
+      </c>
+    </row>
+    <row r="1452" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1452">
+        <v>44632</v>
+      </c>
+      <c r="B1452" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1452" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1452" t="s">
+        <v>1459</v>
+      </c>
+    </row>
+    <row r="1453" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1453">
+        <v>44662</v>
+      </c>
+      <c r="B1453" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1453" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1453" t="s">
+        <v>1460</v>
+      </c>
+    </row>
+    <row r="1454" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1454">
+        <v>44700</v>
+      </c>
+      <c r="B1454" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1454" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1454" t="s">
+        <v>1461</v>
+      </c>
+    </row>
+    <row r="1455" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1455">
+        <v>44711</v>
+      </c>
+      <c r="B1455" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1455" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1455" t="s">
+        <v>1462</v>
+      </c>
+    </row>
+    <row r="1456" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1456">
+        <v>44859</v>
+      </c>
+      <c r="B1456" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1456" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1456" t="s">
+        <v>1463</v>
+      </c>
+    </row>
+    <row r="1457" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1457">
+        <v>46018</v>
+      </c>
+      <c r="B1457" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1457" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1457" t="s">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="1458" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1458">
+        <v>46402</v>
+      </c>
+      <c r="B1458" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1458" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1458" t="s">
+        <v>1465</v>
+      </c>
+    </row>
+    <row r="1459" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1459">
+        <v>46413</v>
+      </c>
+      <c r="B1459" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1459" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1459" t="s">
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="1460" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1460">
+        <v>47141</v>
+      </c>
+      <c r="B1460" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1460" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1460" t="s">
+        <v>1467</v>
+      </c>
+    </row>
+    <row r="1461" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1461">
+        <v>47199</v>
+      </c>
+      <c r="B1461" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1461" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1461" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="1462" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1462">
+        <v>47485</v>
+      </c>
+      <c r="B1462" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1462" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1462" t="s">
+        <v>1469</v>
+      </c>
+    </row>
+    <row r="1463" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1463">
+        <v>48002</v>
+      </c>
+      <c r="B1463" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1463" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1463" t="s">
+        <v>1470</v>
+      </c>
+    </row>
+    <row r="1464" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1464">
+        <v>48003</v>
+      </c>
+      <c r="B1464" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1464" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1464" t="s">
+        <v>1471</v>
+      </c>
+    </row>
+    <row r="1465" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1465">
+        <v>48079</v>
+      </c>
+      <c r="B1465" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1465" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1465" t="s">
+        <v>1472</v>
+      </c>
+    </row>
+    <row r="1466" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1466">
+        <v>48080</v>
+      </c>
+      <c r="B1466" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1466" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1466" t="s">
+        <v>1473</v>
+      </c>
+    </row>
+    <row r="1467" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1467">
+        <v>48634</v>
+      </c>
+      <c r="B1467" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1467" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1467" t="s">
+        <v>1474</v>
+      </c>
+    </row>
+    <row r="1468" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1468">
+        <v>48758</v>
+      </c>
+      <c r="B1468" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1468" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1468" t="s">
+        <v>1475</v>
+      </c>
+    </row>
+    <row r="1469" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1469">
+        <v>48853</v>
+      </c>
+      <c r="B1469" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1469" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1469" t="s">
+        <v>1476</v>
+      </c>
+    </row>
+    <row r="1470" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1470">
+        <v>49407</v>
+      </c>
+      <c r="B1470" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1470" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1470" t="s">
+        <v>1477</v>
+      </c>
+    </row>
+    <row r="1471" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1471">
+        <v>49634</v>
+      </c>
+      <c r="B1471" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1471" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1471" t="s">
+        <v>1478</v>
+      </c>
+    </row>
+    <row r="1472" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1472">
+        <v>51146</v>
+      </c>
+      <c r="B1472" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1472" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1472" t="s">
+        <v>1479</v>
+      </c>
+    </row>
+    <row r="1473" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1473">
+        <v>51558</v>
+      </c>
+      <c r="B1473" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1473" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1473" t="s">
+        <v>1480</v>
+      </c>
+    </row>
+    <row r="1474" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1474">
+        <v>51991</v>
+      </c>
+      <c r="B1474" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1474" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1474" t="s">
+        <v>1481</v>
+      </c>
+    </row>
+    <row r="1475" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1475">
+        <v>52040</v>
+      </c>
+      <c r="B1475" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1475" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1475" t="s">
+        <v>1482</v>
+      </c>
+    </row>
+    <row r="1476" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1476">
+        <v>52187</v>
+      </c>
+      <c r="B1476" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1476" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1476" t="s">
+        <v>1483</v>
+      </c>
+    </row>
+    <row r="1477" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1477">
+        <v>52317</v>
+      </c>
+      <c r="B1477" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1477" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1477" t="s">
+        <v>1484</v>
+      </c>
+    </row>
+    <row r="1478" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1478">
+        <v>52464</v>
+      </c>
+      <c r="B1478" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1478" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1478" t="s">
+        <v>1485</v>
+      </c>
+    </row>
+    <row r="1479" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1479">
+        <v>52465</v>
+      </c>
+      <c r="B1479" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1479" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1479" t="s">
+        <v>1486</v>
+      </c>
+    </row>
+    <row r="1480" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1480">
+        <v>52466</v>
+      </c>
+      <c r="B1480" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1480" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1480" t="s">
+        <v>1487</v>
+      </c>
+    </row>
+    <row r="1481" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1481">
+        <v>52467</v>
+      </c>
+      <c r="B1481" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1481" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1481" t="s">
+        <v>1488</v>
+      </c>
+    </row>
+    <row r="1482" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1482">
+        <v>52631</v>
+      </c>
+      <c r="B1482" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1482" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1482" t="s">
+        <v>1489</v>
+      </c>
+    </row>
+    <row r="1483" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1483">
+        <v>52635</v>
+      </c>
+      <c r="B1483" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1483" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1483" t="s">
+        <v>1490</v>
+      </c>
+    </row>
+    <row r="1484" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1484">
+        <v>52923</v>
+      </c>
+      <c r="B1484" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1484" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1484" t="s">
+        <v>1491</v>
+      </c>
+    </row>
+    <row r="1485" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1485">
+        <v>53488</v>
+      </c>
+      <c r="B1485" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1485" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1485" t="s">
+        <v>1492</v>
+      </c>
+    </row>
+    <row r="1486" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1486">
+        <v>54596</v>
+      </c>
+      <c r="B1486" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1486" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1486" t="s">
+        <v>1493</v>
+      </c>
+    </row>
+    <row r="1487" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1487">
+        <v>55299</v>
+      </c>
+      <c r="B1487" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1487" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1487" t="s">
+        <v>1494</v>
+      </c>
+    </row>
+    <row r="1488" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1488">
+        <v>56209</v>
+      </c>
+      <c r="B1488" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1488" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1488" t="s">
+        <v>1495</v>
+      </c>
+    </row>
+    <row r="1489" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1489">
+        <v>56210</v>
+      </c>
+      <c r="B1489" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1489" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1489" t="s">
+        <v>1496</v>
+      </c>
+    </row>
+    <row r="1490" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1490">
+        <v>56211</v>
+      </c>
+      <c r="B1490" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1490" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1490" t="s">
+        <v>1497</v>
+      </c>
+    </row>
+    <row r="1491" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1491">
+        <v>56220</v>
+      </c>
+      <c r="B1491" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1491" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1491" t="s">
+        <v>1498</v>
+      </c>
+    </row>
+    <row r="1492" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1492">
+        <v>56221</v>
+      </c>
+      <c r="B1492" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1492" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1492" t="s">
+        <v>1499</v>
+      </c>
+    </row>
+    <row r="1493" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1493">
+        <v>56450</v>
+      </c>
+      <c r="B1493" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1493" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1493" t="s">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="1494" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1494">
+        <v>56451</v>
+      </c>
+      <c r="B1494" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1494" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1494" t="s">
+        <v>1501</v>
+      </c>
+    </row>
+    <row r="1495" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1495">
+        <v>56551</v>
+      </c>
+      <c r="B1495" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1495" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1495" t="s">
+        <v>1502</v>
+      </c>
+    </row>
+    <row r="1496" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1496">
+        <v>56552</v>
+      </c>
+      <c r="B1496" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1496" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1496" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="1497" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1497">
+        <v>56553</v>
+      </c>
+      <c r="B1497" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1497" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1497" t="s">
+        <v>1504</v>
+      </c>
+    </row>
+    <row r="1498" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1498">
+        <v>56554</v>
+      </c>
+      <c r="B1498" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1498" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1498" t="s">
+        <v>1505</v>
+      </c>
+    </row>
+    <row r="1499" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1499">
+        <v>56705</v>
+      </c>
+      <c r="B1499" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1499" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1499" t="s">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="1500" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1500">
+        <v>57031</v>
+      </c>
+      <c r="B1500" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1500" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1500" t="s">
+        <v>1507</v>
+      </c>
+    </row>
+    <row r="1501" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1501">
+        <v>57471</v>
+      </c>
+      <c r="B1501" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1501" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1501" t="s">
+        <v>1508</v>
+      </c>
+    </row>
+    <row r="1502" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1502">
+        <v>57656</v>
+      </c>
+      <c r="B1502" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1502" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1502" t="s">
+        <v>1509</v>
+      </c>
+    </row>
+    <row r="1503" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1503">
+        <v>57859</v>
+      </c>
+      <c r="B1503" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1503" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1503" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="1504" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1504">
+        <v>57860</v>
+      </c>
+      <c r="B1504" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1504" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1504" t="s">
+        <v>1511</v>
+      </c>
+    </row>
+    <row r="1505" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1505">
+        <v>58262</v>
+      </c>
+      <c r="B1505" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1505" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1505" t="s">
+        <v>1512</v>
+      </c>
+    </row>
+    <row r="1506" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1506">
+        <v>58263</v>
+      </c>
+      <c r="B1506" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1506" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1506" t="s">
+        <v>1513</v>
+      </c>
+    </row>
+    <row r="1507" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1507">
+        <v>58608</v>
+      </c>
+      <c r="B1507" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1507" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1507" t="s">
+        <v>1514</v>
+      </c>
+    </row>
+    <row r="1508" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1508">
+        <v>58614</v>
+      </c>
+      <c r="B1508" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1508" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1508" t="s">
+        <v>1515</v>
+      </c>
+    </row>
+    <row r="1509" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1509">
+        <v>58626</v>
+      </c>
+      <c r="B1509" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1509" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1509" t="s">
+        <v>1516</v>
+      </c>
+    </row>
+    <row r="1510" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1510">
+        <v>58902</v>
+      </c>
+      <c r="B1510" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1510" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1510" t="s">
+        <v>1517</v>
+      </c>
+    </row>
+    <row r="1511" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1511">
+        <v>59371</v>
+      </c>
+      <c r="B1511" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1511" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1511" t="s">
+        <v>1518</v>
+      </c>
+    </row>
+    <row r="1512" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1512">
+        <v>59372</v>
+      </c>
+      <c r="B1512" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1512" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1512" t="s">
+        <v>1519</v>
+      </c>
+    </row>
+    <row r="1513" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1513">
+        <v>59551</v>
+      </c>
+      <c r="B1513" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1513" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1513" t="s">
+        <v>1520</v>
+      </c>
+    </row>
+    <row r="1514" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1514">
+        <v>59552</v>
+      </c>
+      <c r="B1514" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1514" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1514" t="s">
+        <v>1521</v>
+      </c>
+    </row>
+    <row r="1515" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1515">
+        <v>60703</v>
+      </c>
+      <c r="B1515" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1515" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1515" t="s">
+        <v>1522</v>
+      </c>
+    </row>
+    <row r="1516" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1516">
+        <v>61231</v>
+      </c>
+      <c r="B1516" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1516" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1516" t="s">
+        <v>1523</v>
+      </c>
+    </row>
+    <row r="1517" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1517">
+        <v>61387</v>
+      </c>
+      <c r="B1517" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1517" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1517" t="s">
+        <v>1524</v>
+      </c>
+    </row>
+    <row r="1518" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1518">
+        <v>61470</v>
+      </c>
+      <c r="B1518" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1518" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1518" t="s">
+        <v>1525</v>
+      </c>
+    </row>
+    <row r="1519" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1519">
+        <v>61471</v>
+      </c>
+      <c r="B1519" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1519" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1519" t="s">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="1520" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1520">
+        <v>61472</v>
+      </c>
+      <c r="B1520" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1520" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1520" t="s">
+        <v>1527</v>
+      </c>
+    </row>
+    <row r="1521" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1521">
+        <v>61473</v>
+      </c>
+      <c r="B1521" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1521" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1521" t="s">
+        <v>1528</v>
+      </c>
+    </row>
+    <row r="1522" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1522">
+        <v>61474</v>
+      </c>
+      <c r="B1522" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1522" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1522" t="s">
+        <v>1529</v>
+      </c>
+    </row>
+    <row r="1523" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1523">
+        <v>61503</v>
+      </c>
+      <c r="B1523" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1523" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1523" t="s">
+        <v>1530</v>
+      </c>
+    </row>
+    <row r="1524" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1524">
+        <v>61504</v>
+      </c>
+      <c r="B1524" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1524" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1524" t="s">
+        <v>1531</v>
+      </c>
+    </row>
+    <row r="1525" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1525">
+        <v>61680</v>
+      </c>
+      <c r="B1525" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1525" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1525" t="s">
+        <v>1532</v>
+      </c>
+    </row>
+    <row r="1526" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1526">
+        <v>61691</v>
+      </c>
+      <c r="B1526" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1526" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1526" t="s">
+        <v>1533</v>
+      </c>
+    </row>
+    <row r="1527" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1527">
+        <v>62378</v>
+      </c>
+      <c r="B1527" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1527" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1527" t="s">
+        <v>1534</v>
+      </c>
+    </row>
+    <row r="1528" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1528">
+        <v>62549</v>
+      </c>
+      <c r="B1528" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1528" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1528" t="s">
+        <v>1535</v>
+      </c>
+    </row>
+    <row r="1529" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1529">
+        <v>62562</v>
+      </c>
+      <c r="B1529" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1529" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1529" t="s">
+        <v>1536</v>
+      </c>
+    </row>
+    <row r="1530" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1530">
+        <v>63488</v>
+      </c>
+      <c r="B1530" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1530" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1530" t="s">
+        <v>1537</v>
+      </c>
+    </row>
+    <row r="1531" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1531">
+        <v>63604</v>
+      </c>
+      <c r="B1531" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1531" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1531" t="s">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="1532" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1532">
+        <v>63605</v>
+      </c>
+      <c r="B1532" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1532" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1532" t="s">
+        <v>1539</v>
+      </c>
+    </row>
+    <row r="1533" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1533">
+        <v>64604</v>
+      </c>
+      <c r="B1533" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1533" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1533" t="s">
+        <v>1540</v>
+      </c>
+    </row>
+    <row r="1534" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1534">
+        <v>65516</v>
+      </c>
+      <c r="B1534" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1534" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1534" t="s">
+        <v>1541</v>
+      </c>
+    </row>
+    <row r="1535" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1535">
+        <v>65517</v>
+      </c>
+      <c r="B1535" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1535" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1535" t="s">
+        <v>1542</v>
+      </c>
+    </row>
+    <row r="1536" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1536">
+        <v>66072</v>
+      </c>
+      <c r="B1536" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1536" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1536" t="s">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="1537" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1537">
+        <v>66116</v>
+      </c>
+      <c r="B1537" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1537" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1537" t="s">
+        <v>1544</v>
+      </c>
+    </row>
+    <row r="1538" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1538">
+        <v>66117</v>
+      </c>
+      <c r="B1538" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1538" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1538" t="s">
+        <v>1545</v>
+      </c>
+    </row>
+    <row r="1539" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1539">
+        <v>67366</v>
+      </c>
+      <c r="B1539" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1539" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1539" t="s">
+        <v>1546</v>
+      </c>
+    </row>
+    <row r="1540" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1540">
+        <v>67947</v>
+      </c>
+      <c r="B1540" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1540" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1540" t="s">
+        <v>1547</v>
+      </c>
+    </row>
+    <row r="1541" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1541">
+        <v>69038</v>
+      </c>
+      <c r="B1541" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1541" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1541" t="s">
+        <v>1548</v>
+      </c>
+    </row>
+    <row r="1542" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1542">
+        <v>69039</v>
+      </c>
+      <c r="B1542" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1542" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1542" t="s">
+        <v>1549</v>
+      </c>
+    </row>
+    <row r="1543" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1543">
+        <v>69212</v>
+      </c>
+      <c r="B1543" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1543" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1543" t="s">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="1544" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1544">
+        <v>69312</v>
+      </c>
+      <c r="B1544" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1544" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1544" t="s">
+        <v>1551</v>
+      </c>
+    </row>
+    <row r="1545" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1545">
+        <v>69408</v>
+      </c>
+      <c r="B1545" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1545" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1545" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="1546" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1546">
+        <v>69631</v>
+      </c>
+      <c r="B1546" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1546" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1546" t="s">
+        <v>1553</v>
+      </c>
+    </row>
+    <row r="1547" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1547">
+        <v>69682</v>
+      </c>
+      <c r="B1547" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1547" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1547" t="s">
+        <v>1554</v>
+      </c>
+    </row>
+    <row r="1548" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1548">
+        <v>69683</v>
+      </c>
+      <c r="B1548" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1548" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1548" t="s">
+        <v>1555</v>
+      </c>
+    </row>
+    <row r="1549" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1549">
+        <v>69703</v>
+      </c>
+      <c r="B1549" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1549" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1549" t="s">
+        <v>1556</v>
+      </c>
+    </row>
+    <row r="1550" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1550">
+        <v>70374</v>
+      </c>
+      <c r="B1550" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1550" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1550" t="s">
+        <v>1557</v>
+      </c>
+    </row>
+    <row r="1551" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1551">
+        <v>70816</v>
+      </c>
+      <c r="B1551" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1551" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1551" t="s">
+        <v>1558</v>
+      </c>
+    </row>
+    <row r="1552" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1552">
+        <v>70843</v>
+      </c>
+      <c r="B1552" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1552" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1552" t="s">
+        <v>1559</v>
+      </c>
+    </row>
+    <row r="1553" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1553">
+        <v>70844</v>
+      </c>
+      <c r="B1553" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1553" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1553" t="s">
+        <v>1560</v>
+      </c>
+    </row>
+    <row r="1554" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1554">
+        <v>70845</v>
+      </c>
+      <c r="B1554" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1554" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1554" t="s">
+        <v>1561</v>
+      </c>
+    </row>
+    <row r="1555" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1555">
+        <v>70846</v>
+      </c>
+      <c r="B1555" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1555" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1555" t="s">
+        <v>1562</v>
+      </c>
+    </row>
+    <row r="1556" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1556">
+        <v>71070</v>
+      </c>
+      <c r="B1556" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1556" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1556" t="s">
+        <v>1563</v>
+      </c>
+    </row>
+    <row r="1557" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1557">
+        <v>71071</v>
+      </c>
+      <c r="B1557" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1557" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1557" t="s">
+        <v>1564</v>
+      </c>
+    </row>
+    <row r="1558" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1558">
+        <v>71297</v>
+      </c>
+      <c r="B1558" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1558" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1558" t="s">
+        <v>1565</v>
+      </c>
+    </row>
+    <row r="1559" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1559">
+        <v>71298</v>
+      </c>
+      <c r="B1559" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1559" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1559" t="s">
+        <v>1566</v>
+      </c>
+    </row>
+    <row r="1560" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1560">
+        <v>71299</v>
+      </c>
+      <c r="B1560" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1560" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1560" t="s">
+        <v>1567</v>
+      </c>
+    </row>
+    <row r="1561" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1561">
+        <v>71300</v>
+      </c>
+      <c r="B1561" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1561" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1561" t="s">
+        <v>1568</v>
+      </c>
+    </row>
+    <row r="1562" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1562">
+        <v>71448</v>
+      </c>
+      <c r="B1562" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1562" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1562" t="s">
+        <v>1569</v>
+      </c>
+    </row>
+    <row r="1563" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1563">
+        <v>71561</v>
+      </c>
+      <c r="B1563" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1563" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1563" t="s">
+        <v>1570</v>
+      </c>
+    </row>
+    <row r="1564" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1564">
+        <v>71958</v>
+      </c>
+      <c r="B1564" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1564" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1564" t="s">
+        <v>1571</v>
+      </c>
+    </row>
+    <row r="1565" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1565">
+        <v>72344</v>
+      </c>
+      <c r="B1565" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1565" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1565" t="s">
+        <v>1572</v>
+      </c>
+    </row>
+    <row r="1566" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1566">
+        <v>72345</v>
+      </c>
+      <c r="B1566" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1566" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1566" t="s">
+        <v>1573</v>
+      </c>
+    </row>
+    <row r="1567" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1567">
+        <v>72420</v>
+      </c>
+      <c r="B1567" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1567" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1567" t="s">
+        <v>1574</v>
+      </c>
+    </row>
+    <row r="1568" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1568">
+        <v>72421</v>
+      </c>
+      <c r="B1568" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1568" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1568" t="s">
+        <v>1575</v>
+      </c>
+    </row>
+    <row r="1569" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1569">
+        <v>72553</v>
+      </c>
+      <c r="B1569" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1569" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1569" t="s">
+        <v>1576</v>
+      </c>
+    </row>
+    <row r="1570" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1570">
+        <v>72992</v>
+      </c>
+      <c r="B1570" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1570" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1570" t="s">
+        <v>1577</v>
+      </c>
+    </row>
+    <row r="1571" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1571">
+        <v>73405</v>
+      </c>
+      <c r="B1571" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1571" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1571" t="s">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="1572" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1572">
+        <v>74000</v>
+      </c>
+      <c r="B1572" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1572" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1572" t="s">
+        <v>1579</v>
+      </c>
+    </row>
+    <row r="1573" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1573">
+        <v>74001</v>
+      </c>
+      <c r="B1573" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1573" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1573" t="s">
+        <v>1580</v>
+      </c>
+    </row>
+    <row r="1574" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1574">
+        <v>74002</v>
+      </c>
+      <c r="B1574" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1574" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1574" t="s">
+        <v>1581</v>
+      </c>
+    </row>
+    <row r="1575" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1575">
+        <v>74003</v>
+      </c>
+      <c r="B1575" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1575" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1575" t="s">
+        <v>1582</v>
+      </c>
+    </row>
+    <row r="1576" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1576">
+        <v>74004</v>
+      </c>
+      <c r="B1576" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1576" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1576" t="s">
+        <v>1583</v>
+      </c>
+    </row>
+    <row r="1577" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1577">
+        <v>74005</v>
+      </c>
+      <c r="B1577" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1577" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1577" t="s">
+        <v>1584</v>
+      </c>
+    </row>
+    <row r="1578" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1578">
+        <v>74383</v>
+      </c>
+      <c r="B1578" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1578" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1578" t="s">
+        <v>1585</v>
+      </c>
+    </row>
+    <row r="1579" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1579">
+        <v>74384</v>
+      </c>
+      <c r="B1579" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1579" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1579" t="s">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="1580" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1580">
+        <v>74385</v>
+      </c>
+      <c r="B1580" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1580" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1580" t="s">
+        <v>1587</v>
+      </c>
+    </row>
+    <row r="1581" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1581">
+        <v>77464</v>
+      </c>
+      <c r="B1581" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1581" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1581" t="s">
+        <v>1588</v>
+      </c>
+    </row>
+    <row r="1582" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1582">
+        <v>77465</v>
+      </c>
+      <c r="B1582" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1582" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1582" t="s">
+        <v>1589</v>
+      </c>
+    </row>
+    <row r="1583" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1583">
+        <v>77537</v>
+      </c>
+      <c r="B1583" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1583" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1583" t="s">
+        <v>1590</v>
+      </c>
+    </row>
+    <row r="1584" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1584">
+        <v>77538</v>
+      </c>
+      <c r="B1584" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1584" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1584" t="s">
+        <v>1591</v>
+      </c>
+    </row>
+    <row r="1585" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1585">
+        <v>77939</v>
+      </c>
+      <c r="B1585" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1585" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1585" t="s">
+        <v>1592</v>
+      </c>
+    </row>
+    <row r="1586" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1586">
+        <v>77940</v>
+      </c>
+      <c r="B1586" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1586" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1586" t="s">
+        <v>1593</v>
+      </c>
+    </row>
+    <row r="1587" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1587">
+        <v>78674</v>
+      </c>
+      <c r="B1587" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1587" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1587" t="s">
+        <v>1594</v>
+      </c>
+    </row>
+    <row r="1588" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1588">
+        <v>79284</v>
+      </c>
+      <c r="B1588" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1588" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1588" t="s">
+        <v>1595</v>
+      </c>
+    </row>
+    <row r="1589" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1589">
+        <v>79285</v>
+      </c>
+      <c r="B1589" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1589" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1589" t="s">
+        <v>1596</v>
+      </c>
+    </row>
+    <row r="1590" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1590">
+        <v>79753</v>
+      </c>
+      <c r="B1590" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1590" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1590" t="s">
+        <v>1597</v>
+      </c>
+    </row>
+    <row r="1591" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1591">
+        <v>80718</v>
+      </c>
+      <c r="B1591" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1591" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1591" t="s">
+        <v>1598</v>
+      </c>
+    </row>
+    <row r="1592" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1592">
+        <v>80719</v>
+      </c>
+      <c r="B1592" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1592" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1592" t="s">
+        <v>1599</v>
+      </c>
+    </row>
+    <row r="1593" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1593">
+        <v>80858</v>
+      </c>
+      <c r="B1593" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1593" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1593" t="s">
+        <v>1600</v>
+      </c>
+    </row>
+    <row r="1594" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1594">
+        <v>80859</v>
+      </c>
+      <c r="B1594" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1594" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1594" t="s">
+        <v>1601</v>
+      </c>
+    </row>
+    <row r="1595" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1595">
+        <v>80965</v>
+      </c>
+      <c r="B1595" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1595" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1595" t="s">
+        <v>1602</v>
+      </c>
+    </row>
+    <row r="1596" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1596">
+        <v>81071</v>
+      </c>
+      <c r="B1596" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1596" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1596" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="1597" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1597">
+        <v>81072</v>
+      </c>
+      <c r="B1597" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1597" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1597" t="s">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="1598" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1598">
+        <v>81073</v>
+      </c>
+      <c r="B1598" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1598" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1598" t="s">
+        <v>1605</v>
+      </c>
+    </row>
+    <row r="1599" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1599">
+        <v>81190</v>
+      </c>
+      <c r="B1599" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1599" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1599" t="s">
+        <v>1606</v>
+      </c>
+    </row>
+    <row r="1600" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1600">
+        <v>81776</v>
+      </c>
+      <c r="B1600" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1600" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1600" t="s">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="1601" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1601">
+        <v>81777</v>
+      </c>
+      <c r="B1601" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1601" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1601" t="s">
+        <v>1608</v>
+      </c>
+    </row>
+    <row r="1602" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1602">
+        <v>81778</v>
+      </c>
+      <c r="B1602" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1602" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1602" t="s">
+        <v>1609</v>
+      </c>
+    </row>
+    <row r="1603" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1603">
+        <v>81779</v>
+      </c>
+      <c r="B1603" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1603" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1603" t="s">
+        <v>1610</v>
+      </c>
+    </row>
+    <row r="1604" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1604">
+        <v>81976</v>
+      </c>
+      <c r="B1604" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1604" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1604" t="s">
+        <v>1611</v>
+      </c>
+    </row>
+    <row r="1605" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1605">
+        <v>81977</v>
+      </c>
+      <c r="B1605" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1605" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1605" t="s">
+        <v>1612</v>
+      </c>
+    </row>
+    <row r="1606" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1606">
+        <v>82121</v>
+      </c>
+      <c r="B1606" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1606" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1606" t="s">
+        <v>1613</v>
+      </c>
+    </row>
+    <row r="1607" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1607">
+        <v>82245</v>
+      </c>
+      <c r="B1607" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1607" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1607" t="s">
+        <v>1614</v>
+      </c>
+    </row>
+    <row r="1608" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1608">
+        <v>82413</v>
+      </c>
+      <c r="B1608" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1608" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1608" t="s">
+        <v>1615</v>
+      </c>
+    </row>
+    <row r="1609" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1609">
+        <v>82766</v>
+      </c>
+      <c r="B1609" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1609" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1609" t="s">
+        <v>1616</v>
+      </c>
+    </row>
+    <row r="1610" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1610">
+        <v>82767</v>
+      </c>
+      <c r="B1610" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1610" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1610" t="s">
+        <v>1617</v>
+      </c>
+    </row>
+    <row r="1611" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1611">
+        <v>82914</v>
+      </c>
+      <c r="B1611" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1611" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1611" t="s">
+        <v>1618</v>
+      </c>
+    </row>
+    <row r="1612" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1612">
+        <v>82915</v>
+      </c>
+      <c r="B1612" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1612" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1612" t="s">
+        <v>1619</v>
+      </c>
+    </row>
+    <row r="1613" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1613">
+        <v>83194</v>
+      </c>
+      <c r="B1613" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1613" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1613" t="s">
+        <v>1620</v>
+      </c>
+    </row>
+    <row r="1614" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1614">
+        <v>83468</v>
+      </c>
+      <c r="B1614" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1614" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1614" t="s">
+        <v>1621</v>
+      </c>
+    </row>
+    <row r="1615" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1615">
+        <v>84021</v>
+      </c>
+      <c r="B1615" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1615" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1615" t="s">
+        <v>1622</v>
+      </c>
+    </row>
+    <row r="1616" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1616">
+        <v>84022</v>
+      </c>
+      <c r="B1616" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1616" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1616" t="s">
+        <v>1623</v>
+      </c>
+    </row>
+    <row r="1617" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1617">
+        <v>84194</v>
+      </c>
+      <c r="B1617" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1617" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1617" t="s">
+        <v>1624</v>
+      </c>
+    </row>
+    <row r="1618" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1618">
+        <v>84378</v>
+      </c>
+      <c r="B1618" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1618" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1618" t="s">
+        <v>1625</v>
+      </c>
+    </row>
+    <row r="1619" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1619">
+        <v>84471</v>
+      </c>
+      <c r="B1619" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1619" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1619" t="s">
+        <v>1626</v>
+      </c>
+    </row>
+    <row r="1620" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1620">
+        <v>84472</v>
+      </c>
+      <c r="B1620" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1620" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1620" t="s">
+        <v>1627</v>
+      </c>
+    </row>
+    <row r="1621" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1621">
+        <v>84473</v>
+      </c>
+      <c r="B1621" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1621" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1621" t="s">
+        <v>1628</v>
+      </c>
+    </row>
+    <row r="1622" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1622">
+        <v>84499</v>
+      </c>
+      <c r="B1622" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1622" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1622" t="s">
+        <v>1629</v>
+      </c>
+    </row>
+    <row r="1623" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1623">
+        <v>84504</v>
+      </c>
+      <c r="B1623" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1623" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1623" t="s">
+        <v>1630</v>
+      </c>
+    </row>
+    <row r="1624" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1624">
+        <v>84567</v>
+      </c>
+      <c r="B1624" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1624" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1624" t="s">
+        <v>1631</v>
+      </c>
+    </row>
+    <row r="1625" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1625">
+        <v>84568</v>
+      </c>
+      <c r="B1625" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1625" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1625" t="s">
+        <v>1632</v>
+      </c>
+    </row>
+    <row r="1626" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1626">
+        <v>84689</v>
+      </c>
+      <c r="B1626" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1626" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1626" t="s">
+        <v>1633</v>
+      </c>
+    </row>
+    <row r="1627" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1627">
+        <v>84690</v>
+      </c>
+      <c r="B1627" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1627" t="s">
+        <v>1634</v>
+      </c>
+      <c r="D1627" t="s">
+        <v>1635</v>
+      </c>
+    </row>
+    <row r="1628" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1628">
+        <v>84701</v>
+      </c>
+      <c r="B1628" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1628" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1628" t="s">
+        <v>1636</v>
+      </c>
+    </row>
+    <row r="1629" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1629">
+        <v>84719</v>
+      </c>
+      <c r="B1629" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1629" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1629" t="s">
+        <v>1637</v>
+      </c>
+    </row>
+    <row r="1630" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1630">
+        <v>84720</v>
+      </c>
+      <c r="B1630" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1630" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1630" t="s">
+        <v>1638</v>
+      </c>
+    </row>
+    <row r="1631" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1631">
+        <v>84861</v>
+      </c>
+      <c r="B1631" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1631" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1631" t="s">
+        <v>1639</v>
+      </c>
+    </row>
+    <row r="1632" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1632">
+        <v>84862</v>
+      </c>
+      <c r="B1632" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1632" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1632" t="s">
+        <v>1640</v>
+      </c>
+    </row>
+    <row r="1633" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1633">
+        <v>85279</v>
+      </c>
+      <c r="B1633" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1633" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1633" t="s">
+        <v>1641</v>
+      </c>
+    </row>
+    <row r="1634" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1634">
+        <v>85309</v>
+      </c>
+      <c r="B1634" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1634" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1634" t="s">
+        <v>1642</v>
+      </c>
+    </row>
+    <row r="1635" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1635">
+        <v>85310</v>
+      </c>
+      <c r="B1635" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1635" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1635" t="s">
+        <v>1643</v>
+      </c>
+    </row>
+    <row r="1636" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1636">
+        <v>85374</v>
+      </c>
+      <c r="B1636" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1636" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1636" t="s">
+        <v>1644</v>
+      </c>
+    </row>
+    <row r="1637" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1637">
+        <v>85375</v>
+      </c>
+      <c r="B1637" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1637" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1637" t="s">
+        <v>1645</v>
+      </c>
+    </row>
+    <row r="1638" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1638">
+        <v>85425</v>
+      </c>
+      <c r="B1638" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1638" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1638" t="s">
+        <v>1646</v>
+      </c>
+    </row>
+    <row r="1639" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1639">
+        <v>85705</v>
+      </c>
+      <c r="B1639" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1639" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1639" t="s">
+        <v>1647</v>
+      </c>
+    </row>
+    <row r="1640" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1640">
+        <v>85728</v>
+      </c>
+      <c r="B1640" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1640" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1640" t="s">
+        <v>1648</v>
+      </c>
+    </row>
+    <row r="1641" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1641">
+        <v>85834</v>
+      </c>
+      <c r="B1641" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1641" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1641" t="s">
+        <v>1649</v>
+      </c>
+    </row>
+    <row r="1642" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1642">
+        <v>85839</v>
+      </c>
+      <c r="B1642" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1642" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1642" t="s">
+        <v>1650</v>
+      </c>
+    </row>
+    <row r="1643" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1643">
+        <v>85993</v>
+      </c>
+      <c r="B1643" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1643" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1643" t="s">
+        <v>1651</v>
+      </c>
+    </row>
+    <row r="1644" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1644">
+        <v>86174</v>
+      </c>
+      <c r="B1644" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1644" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1644" t="s">
+        <v>1652</v>
+      </c>
+    </row>
+    <row r="1645" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1645">
+        <v>86175</v>
+      </c>
+      <c r="B1645" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1645" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1645" t="s">
+        <v>1653</v>
+      </c>
+    </row>
+    <row r="1646" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1646">
+        <v>86176</v>
+      </c>
+      <c r="B1646" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1646" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1646" t="s">
+        <v>1654</v>
+      </c>
+    </row>
+    <row r="1647" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1647">
+        <v>86327</v>
+      </c>
+      <c r="B1647" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1647" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1647" t="s">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="1648" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1648">
+        <v>86372</v>
+      </c>
+      <c r="B1648" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1648" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1648" t="s">
+        <v>1656</v>
+      </c>
+    </row>
+    <row r="1649" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1649">
+        <v>86373</v>
+      </c>
+      <c r="B1649" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1649" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1649" t="s">
+        <v>1657</v>
+      </c>
+    </row>
+    <row r="1650" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1650">
+        <v>86379</v>
+      </c>
+      <c r="B1650" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1650" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1650" t="s">
+        <v>1658</v>
+      </c>
+    </row>
+    <row r="1651" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1651">
+        <v>86403</v>
+      </c>
+      <c r="B1651" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1651" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1651" t="s">
+        <v>1659</v>
+      </c>
+    </row>
+    <row r="1652" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1652">
+        <v>86404</v>
+      </c>
+      <c r="B1652" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1652" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1652" t="s">
+        <v>1660</v>
+      </c>
+    </row>
+    <row r="1653" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1653">
+        <v>86405</v>
+      </c>
+      <c r="B1653" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1653" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1653" t="s">
+        <v>1661</v>
+      </c>
+    </row>
+    <row r="1654" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1654">
+        <v>86525</v>
+      </c>
+      <c r="B1654" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1654" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1654" t="s">
+        <v>1662</v>
+      </c>
+    </row>
+    <row r="1655" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1655">
+        <v>86528</v>
+      </c>
+      <c r="B1655" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1655" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1655" t="s">
+        <v>1663</v>
+      </c>
+    </row>
+    <row r="1656" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1656">
+        <v>86533</v>
+      </c>
+      <c r="B1656" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1656" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1656" t="s">
+        <v>1664</v>
+      </c>
+    </row>
+    <row r="1657" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1657">
+        <v>86534</v>
+      </c>
+      <c r="B1657" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1657" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1657" t="s">
+        <v>1665</v>
+      </c>
+    </row>
+    <row r="1658" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1658">
+        <v>86545</v>
+      </c>
+      <c r="B1658" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1658" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1658" t="s">
+        <v>1666</v>
+      </c>
+    </row>
+    <row r="1659" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1659">
+        <v>86546</v>
+      </c>
+      <c r="B1659" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1659" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1659" t="s">
+        <v>1667</v>
+      </c>
+    </row>
+    <row r="1660" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1660">
+        <v>86547</v>
+      </c>
+      <c r="B1660" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1660" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1660" t="s">
+        <v>1668</v>
+      </c>
+    </row>
+    <row r="1661" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1661">
+        <v>86633</v>
+      </c>
+      <c r="B1661" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1661" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1661" t="s">
+        <v>1669</v>
+      </c>
+    </row>
+    <row r="1662" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1662">
+        <v>86750</v>
+      </c>
+      <c r="B1662" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1662" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1662" t="s">
+        <v>1670</v>
+      </c>
+    </row>
+    <row r="1663" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1663">
+        <v>86751</v>
+      </c>
+      <c r="B1663" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1663" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1663" t="s">
+        <v>1671</v>
+      </c>
+    </row>
+    <row r="1664" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1664">
+        <v>86771</v>
+      </c>
+      <c r="B1664" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1664" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1664" t="s">
+        <v>1672</v>
+      </c>
+    </row>
+    <row r="1665" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1665">
+        <v>86772</v>
+      </c>
+      <c r="B1665" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1665" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1665" t="s">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="1666" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1666">
+        <v>86814</v>
+      </c>
+      <c r="B1666" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1666" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1666" t="s">
+        <v>1674</v>
+      </c>
+    </row>
+    <row r="1667" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1667">
+        <v>86916</v>
+      </c>
+      <c r="B1667" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1667" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1667" t="s">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="1668" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1668">
+        <v>86917</v>
+      </c>
+      <c r="B1668" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1668" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1668" t="s">
+        <v>1676</v>
+      </c>
+    </row>
+    <row r="1669" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1669">
+        <v>86918</v>
+      </c>
+      <c r="B1669" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1669" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1669" t="s">
+        <v>1677</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
fix(ui): fix filter issue
</commit_message>
<xml_diff>
--- a/apps/backend/excel-data/issuereturn_library_migration.xlsx
+++ b/apps/backend/excel-data/issuereturn_library_migration.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5008" uniqueCount="1678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5098" uniqueCount="1708">
   <si>
     <t>legacy_id</t>
   </si>
@@ -5046,6 +5046,96 @@
   </si>
   <si>
     <t>2026-05-11T08:00:15.126Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:00:52.949Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:01:30.230Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:01:37.829Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:01:42.079Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:01:54.274Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:01:56.857Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:08.990Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:10.729Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:12.261Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:13.850Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:21.129Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:35.592Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:42.941Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:49.287Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:51.584Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:53.209Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:54.418Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:02:55.487Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:03:02.392Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:03:15.135Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:03:22.745Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:03:29.350Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:03:38.296Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:03:45.798Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:03:54.169Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:03:56.217Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:03:57.481Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:03:59.465Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:04:00.978Z</t>
+  </si>
+  <si>
+    <t>2026-05-11T08:04:02.152Z</t>
   </si>
 </sst>
 </file>
@@ -5426,7 +5516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D1669"/>
+  <dimension ref="A1:D1699"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -28795,6 +28885,426 @@
         <v>1677</v>
       </c>
     </row>
+    <row r="1670" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1670">
+        <v>86919</v>
+      </c>
+      <c r="B1670" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1670" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1670" t="s">
+        <v>1678</v>
+      </c>
+    </row>
+    <row r="1671" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1671">
+        <v>87072</v>
+      </c>
+      <c r="B1671" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1671" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1671" t="s">
+        <v>1679</v>
+      </c>
+    </row>
+    <row r="1672" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1672">
+        <v>87365</v>
+      </c>
+      <c r="B1672" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1672" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1672" t="s">
+        <v>1680</v>
+      </c>
+    </row>
+    <row r="1673" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1673">
+        <v>87366</v>
+      </c>
+      <c r="B1673" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1673" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1673" t="s">
+        <v>1681</v>
+      </c>
+    </row>
+    <row r="1674" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1674">
+        <v>87405</v>
+      </c>
+      <c r="B1674" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1674" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1674" t="s">
+        <v>1682</v>
+      </c>
+    </row>
+    <row r="1675" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1675">
+        <v>87406</v>
+      </c>
+      <c r="B1675" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1675" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1675" t="s">
+        <v>1683</v>
+      </c>
+    </row>
+    <row r="1676" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1676">
+        <v>87407</v>
+      </c>
+      <c r="B1676" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1676" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1676" t="s">
+        <v>1684</v>
+      </c>
+    </row>
+    <row r="1677" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1677">
+        <v>87532</v>
+      </c>
+      <c r="B1677" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1677" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1677" t="s">
+        <v>1685</v>
+      </c>
+    </row>
+    <row r="1678" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1678">
+        <v>87533</v>
+      </c>
+      <c r="B1678" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1678" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1678" t="s">
+        <v>1686</v>
+      </c>
+    </row>
+    <row r="1679" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1679">
+        <v>87534</v>
+      </c>
+      <c r="B1679" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1679" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1679" t="s">
+        <v>1687</v>
+      </c>
+    </row>
+    <row r="1680" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1680">
+        <v>87558</v>
+      </c>
+      <c r="B1680" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1680" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1680" t="s">
+        <v>1688</v>
+      </c>
+    </row>
+    <row r="1681" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1681">
+        <v>87580</v>
+      </c>
+      <c r="B1681" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1681" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1681" t="s">
+        <v>1689</v>
+      </c>
+    </row>
+    <row r="1682" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1682">
+        <v>87674</v>
+      </c>
+      <c r="B1682" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1682" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1682" t="s">
+        <v>1690</v>
+      </c>
+    </row>
+    <row r="1683" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1683">
+        <v>87731</v>
+      </c>
+      <c r="B1683" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1683" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1683" t="s">
+        <v>1691</v>
+      </c>
+    </row>
+    <row r="1684" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1684">
+        <v>87745</v>
+      </c>
+      <c r="B1684" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1684" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1684" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="1685" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1685">
+        <v>87746</v>
+      </c>
+      <c r="B1685" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1685" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1685" t="s">
+        <v>1693</v>
+      </c>
+    </row>
+    <row r="1686" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1686">
+        <v>87747</v>
+      </c>
+      <c r="B1686" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1686" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1686" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="1687" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1687">
+        <v>87748</v>
+      </c>
+      <c r="B1687" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1687" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1687" t="s">
+        <v>1695</v>
+      </c>
+    </row>
+    <row r="1688" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1688">
+        <v>87753</v>
+      </c>
+      <c r="B1688" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1688" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1688" t="s">
+        <v>1696</v>
+      </c>
+    </row>
+    <row r="1689" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1689">
+        <v>87800</v>
+      </c>
+      <c r="B1689" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1689" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1689" t="s">
+        <v>1697</v>
+      </c>
+    </row>
+    <row r="1690" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1690">
+        <v>87801</v>
+      </c>
+      <c r="B1690" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1690" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1690" t="s">
+        <v>1698</v>
+      </c>
+    </row>
+    <row r="1691" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1691">
+        <v>87802</v>
+      </c>
+      <c r="B1691" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1691" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1691" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="1692" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1692">
+        <v>88131</v>
+      </c>
+      <c r="B1692" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1692" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1692" t="s">
+        <v>1700</v>
+      </c>
+    </row>
+    <row r="1693" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1693">
+        <v>88132</v>
+      </c>
+      <c r="B1693" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1693" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1693" t="s">
+        <v>1701</v>
+      </c>
+    </row>
+    <row r="1694" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1694">
+        <v>88280</v>
+      </c>
+      <c r="B1694" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1694" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1694" t="s">
+        <v>1702</v>
+      </c>
+    </row>
+    <row r="1695" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1695">
+        <v>88317</v>
+      </c>
+      <c r="B1695" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1695" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1695" t="s">
+        <v>1703</v>
+      </c>
+    </row>
+    <row r="1696" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1696">
+        <v>88318</v>
+      </c>
+      <c r="B1696" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1696" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1696" t="s">
+        <v>1704</v>
+      </c>
+    </row>
+    <row r="1697" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1697">
+        <v>88373</v>
+      </c>
+      <c r="B1697" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1697" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1697" t="s">
+        <v>1705</v>
+      </c>
+    </row>
+    <row r="1698" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1698">
+        <v>88381</v>
+      </c>
+      <c r="B1698" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1698" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1698" t="s">
+        <v>1706</v>
+      </c>
+    </row>
+    <row r="1699" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1699">
+        <v>88382</v>
+      </c>
+      <c r="B1699" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1699" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1699" t="s">
+        <v>1707</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>